<commit_message>
Atulizando preco dia 12/10
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodosLibanes.xlsx
+++ b/data/ProdutosFomatodosLibanes.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3740" uniqueCount="1130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3744" uniqueCount="1130">
   <si>
     <t>produto_grupo</t>
   </si>
@@ -4267,10 +4267,10 @@
         <v>29</v>
       </c>
       <c r="G16" s="3">
-        <v>155</v>
+        <v>130</v>
       </c>
       <c r="H16" s="3">
-        <v>160</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5354,7 +5354,7 @@
         <v>14</v>
       </c>
       <c r="H18" s="3">
-        <f>MROUND(G17*1.03, 0.5)</f>
+        <f>MROUND(G18*1.03, 0.5)</f>
       </c>
     </row>
     <row r="19" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5380,7 +5380,7 @@
         <v>55</v>
       </c>
       <c r="H19" s="3">
-        <f>MROUND(G18*1.03, 0.5)</f>
+        <f>MROUND(G19*1.03, 0.5)</f>
       </c>
     </row>
     <row r="20" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5406,7 +5406,7 @@
         <v>530</v>
       </c>
       <c r="H20" s="3">
-        <f>MROUND(G19*1.03, 0.5)</f>
+        <f>MROUND(G20*1.03, 0.5)</f>
       </c>
     </row>
     <row r="21" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5432,7 +5432,7 @@
         <v>275</v>
       </c>
       <c r="H21" s="3">
-        <f>MROUND(G20*1.03, 0.5)</f>
+        <f>MROUND(G21*1.03, 0.5)</f>
       </c>
     </row>
     <row r="22" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5458,7 +5458,7 @@
         <v>940</v>
       </c>
       <c r="H22" s="3">
-        <f>MROUND(G21*1.03, 0.5)</f>
+        <f>MROUND(G22*1.03, 0.5)</f>
       </c>
     </row>
     <row r="23" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5484,7 +5484,7 @@
         <v>237</v>
       </c>
       <c r="H23" s="3">
-        <f>MROUND(G22*1.03, 0.5)</f>
+        <f>MROUND(G23*1.03, 0.5)</f>
       </c>
     </row>
     <row r="24" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5510,7 +5510,7 @@
         <v>140</v>
       </c>
       <c r="H24" s="3">
-        <f>MROUND(G23*1.03, 0.5)</f>
+        <f>MROUND(G24*1.03, 0.5)</f>
       </c>
     </row>
     <row r="25" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5536,7 +5536,7 @@
         <v>140</v>
       </c>
       <c r="H25" s="3">
-        <f>MROUND(G24*1.03, 0.5)</f>
+        <f>MROUND(G25*1.03, 0.5)</f>
       </c>
     </row>
     <row r="26" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5562,7 +5562,7 @@
         <v>209</v>
       </c>
       <c r="H26" s="3">
-        <f>MROUND(G25*1.03, 0.5)</f>
+        <f>MROUND(G26*1.03, 0.5)</f>
       </c>
     </row>
     <row r="27" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5588,7 +5588,7 @@
         <v>119</v>
       </c>
       <c r="H27" s="3">
-        <f>MROUND(G26*1.03, 0.5)</f>
+        <f>MROUND(G27*1.03, 0.5)</f>
       </c>
     </row>
     <row r="28" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5614,7 +5614,7 @@
         <v>119</v>
       </c>
       <c r="H28" s="3">
-        <f>MROUND(G27*1.03, 0.5)</f>
+        <f>MROUND(G28*1.03, 0.5)</f>
       </c>
     </row>
     <row r="29" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5640,7 +5640,7 @@
         <v>158.5</v>
       </c>
       <c r="H29" s="3">
-        <f>MROUND(G28*1.03, 0.5)</f>
+        <f>MROUND(G29*1.03, 0.5)</f>
       </c>
     </row>
     <row r="30" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5666,7 +5666,7 @@
         <v>119</v>
       </c>
       <c r="H30" s="3">
-        <f>MROUND(G29*1.03, 0.5)</f>
+        <f>MROUND(G30*1.03, 0.5)</f>
       </c>
     </row>
     <row r="31" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5692,7 +5692,7 @@
         <v>158.5</v>
       </c>
       <c r="H31" s="3">
-        <f>MROUND(G30*1.03, 0.5)</f>
+        <f>MROUND(G31*1.03, 0.5)</f>
       </c>
     </row>
     <row r="32" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5718,7 +5718,7 @@
         <v>153.5</v>
       </c>
       <c r="H32" s="3">
-        <f>MROUND(G31*1.03, 0.5)</f>
+        <f>MROUND(G32*1.03, 0.5)</f>
       </c>
     </row>
     <row r="33" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>177</v>
       </c>
       <c r="H33" s="3">
-        <f>MROUND(G32*1.03, 0.5)</f>
+        <f>MROUND(G33*1.03, 0.5)</f>
       </c>
     </row>
     <row r="34" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5770,7 +5770,7 @@
         <v>38.5</v>
       </c>
       <c r="H34" s="3">
-        <f>MROUND(G33*1.03, 0.5)</f>
+        <f>MROUND(G34*1.03, 0.5)</f>
       </c>
     </row>
     <row r="35" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5796,7 +5796,7 @@
         <v>177</v>
       </c>
       <c r="H35" s="3">
-        <f>MROUND(G34*1.03, 0.5)</f>
+        <f>MROUND(G35*1.03, 0.5)</f>
       </c>
     </row>
     <row r="36" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5822,7 +5822,7 @@
         <v>38.5</v>
       </c>
       <c r="H36" s="3">
-        <f>MROUND(G35*1.03, 0.5)</f>
+        <f>MROUND(G36*1.03, 0.5)</f>
       </c>
     </row>
     <row r="37" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5848,7 +5848,7 @@
         <v>164</v>
       </c>
       <c r="H37" s="3">
-        <f>MROUND(G36*1.03, 0.5)</f>
+        <f>MROUND(G37*1.03, 0.5)</f>
       </c>
     </row>
     <row r="38" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5874,7 +5874,7 @@
         <v>125</v>
       </c>
       <c r="H38" s="3">
-        <f>MROUND(G37*1.03, 0.5)</f>
+        <f>MROUND(G38*1.03, 0.5)</f>
       </c>
     </row>
     <row r="39" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5900,7 +5900,7 @@
         <v>28</v>
       </c>
       <c r="H39" s="3">
-        <f>MROUND(G38*1.03, 0.5)</f>
+        <f>MROUND(G39*1.03, 0.5)</f>
       </c>
     </row>
   </sheetData>
@@ -6310,7 +6310,7 @@
         <v>280</v>
       </c>
       <c r="H15" s="3">
-        <f>MROUND(G14*1.03, 0.5)</f>
+        <f>MROUND(G15*1.03, 0.5)</f>
       </c>
     </row>
     <row r="16" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6336,7 +6336,7 @@
         <v>580</v>
       </c>
       <c r="H16" s="3">
-        <f>MROUND(G15*1.03, 0.5)</f>
+        <f>MROUND(G16*1.03, 0.5)</f>
       </c>
     </row>
     <row r="17" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6362,7 +6362,7 @@
         <v>290</v>
       </c>
       <c r="H17" s="3">
-        <f>MROUND(G16*1.03, 0.5)</f>
+        <f>MROUND(G17*1.03, 0.5)</f>
       </c>
     </row>
     <row r="18" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6388,7 +6388,7 @@
         <v>675.5</v>
       </c>
       <c r="H18" s="3">
-        <f>MROUND(G17*1.03, 0.5)</f>
+        <f>MROUND(G18*1.03, 0.5)</f>
       </c>
     </row>
     <row r="19" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6414,7 +6414,7 @@
         <v>337.5</v>
       </c>
       <c r="H19" s="3">
-        <f>MROUND(G18*1.03, 0.5)</f>
+        <f>MROUND(G19*1.03, 0.5)</f>
       </c>
     </row>
     <row r="20" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>275</v>
       </c>
       <c r="H20" s="3">
-        <f>MROUND(G19*1.03, 0.5)</f>
+        <f>MROUND(G20*1.03, 0.5)</f>
       </c>
     </row>
     <row r="21" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6466,7 +6466,7 @@
         <v>245</v>
       </c>
       <c r="H21" s="3">
-        <f>MROUND(G20*1.03, 0.5)</f>
+        <f>MROUND(G21*1.03, 0.5)</f>
       </c>
     </row>
     <row r="22" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6492,7 +6492,7 @@
         <v>147</v>
       </c>
       <c r="H22" s="3">
-        <f>MROUND(G21*1.03, 0.5)</f>
+        <f>MROUND(G22*1.03, 0.5)</f>
       </c>
     </row>
     <row r="23" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6518,7 +6518,7 @@
         <v>142</v>
       </c>
       <c r="H23" s="3">
-        <f>MROUND(G22*1.03, 0.5)</f>
+        <f>MROUND(G23*1.03, 0.5)</f>
       </c>
     </row>
     <row r="24" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6541,10 +6541,10 @@
         <v>29</v>
       </c>
       <c r="G24" s="3">
-        <v>340</v>
+        <v>400</v>
       </c>
       <c r="H24" s="3">
-        <f>MROUND(G23*1.03, 0.5)</f>
+        <f>MROUND(G24*1.03, 0.5)</f>
       </c>
     </row>
     <row r="25" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6567,10 +6567,10 @@
         <v>29</v>
       </c>
       <c r="G25" s="3">
-        <v>155</v>
+        <v>130</v>
       </c>
       <c r="H25" s="3">
-        <f>MROUND(G24*1.03, 0.5)</f>
+        <f>MROUND(G25*1.03, 0.5)</f>
       </c>
     </row>
   </sheetData>
@@ -9260,7 +9260,7 @@
         <v>11</v>
       </c>
       <c r="G67" s="3">
-        <v>900</v>
+        <v>975</v>
       </c>
       <c r="H67" s="3">
         <f>MROUND(G67*1.03, 0.5)</f>
@@ -9286,7 +9286,7 @@
         <v>12</v>
       </c>
       <c r="G68" s="3">
-        <v>182</v>
+        <v>198.5</v>
       </c>
       <c r="H68" s="3">
         <f>MROUND(G68*1.03, 0.5)</f>
@@ -9783,7 +9783,7 @@
         <v>430</v>
       </c>
       <c r="H87" s="3">
-        <f>MROUND(G88*1.03, 0.5)</f>
+        <f>MROUND(G87*1.03, 0.5)</f>
       </c>
     </row>
     <row r="88" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9809,7 +9809,7 @@
         <v>43</v>
       </c>
       <c r="H88" s="3">
-        <f>MROUND(G89*1.03, 0.5)</f>
+        <f>MROUND(G88*1.03, 0.5)</f>
       </c>
     </row>
     <row r="89" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9835,7 +9835,7 @@
         <v>350</v>
       </c>
       <c r="H89" s="3">
-        <f>MROUND(G90*1.03, 0.5)</f>
+        <f>MROUND(G89*1.03, 0.5)</f>
       </c>
     </row>
     <row r="90" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9861,7 +9861,7 @@
         <v>72</v>
       </c>
       <c r="H90" s="3">
-        <f>MROUND(G91*1.03, 0.5)</f>
+        <f>MROUND(G90*1.03, 0.5)</f>
       </c>
     </row>
     <row r="91" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9887,7 +9887,7 @@
         <v>158</v>
       </c>
       <c r="H91" s="3">
-        <f>MROUND(G92*1.03, 0.5)</f>
+        <f>MROUND(G91*1.03, 0.5)</f>
       </c>
     </row>
     <row r="92" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9913,7 +9913,7 @@
         <v>216.5</v>
       </c>
       <c r="H92" s="3">
-        <f>MROUND(G93*1.03, 0.5)</f>
+        <f>MROUND(G92*1.03, 0.5)</f>
       </c>
     </row>
     <row r="93" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9939,7 +9939,7 @@
         <v>132</v>
       </c>
       <c r="H93" s="3">
-        <f>MROUND(G94*1.03, 0.5)</f>
+        <f>MROUND(G93*1.03, 0.5)</f>
       </c>
     </row>
     <row r="94" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9965,7 +9965,7 @@
         <v>132</v>
       </c>
       <c r="H94" s="3">
-        <f>MROUND(G95*1.03, 0.5)</f>
+        <f>MROUND(G94*1.03, 0.5)</f>
       </c>
     </row>
     <row r="95" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9991,7 +9991,7 @@
         <v>375</v>
       </c>
       <c r="H95" s="3">
-        <f>MROUND(G96*1.03, 0.5)</f>
+        <f>MROUND(G95*1.03, 0.5)</f>
       </c>
     </row>
     <row r="96" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10017,7 +10017,7 @@
         <v>150</v>
       </c>
       <c r="H96" s="3">
-        <f>MROUND(G97*1.03, 0.5)</f>
+        <f>MROUND(G96*1.03, 0.5)</f>
       </c>
     </row>
     <row r="97" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10043,7 +10043,7 @@
         <v>46</v>
       </c>
       <c r="H97" s="3">
-        <f>MROUND(G98*1.03, 0.5)</f>
+        <f>MROUND(G97*1.03, 0.5)</f>
       </c>
     </row>
     <row r="98" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10069,7 +10069,7 @@
         <v>350</v>
       </c>
       <c r="H98" s="3">
-        <f>MROUND(G99*1.03, 0.5)</f>
+        <f>MROUND(G98*1.03, 0.5)</f>
       </c>
     </row>
     <row r="99" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10095,7 +10095,7 @@
         <v>178.5</v>
       </c>
       <c r="H99" s="3">
-        <f>MROUND(G100*1.03, 0.5)</f>
+        <f>MROUND(G99*1.03, 0.5)</f>
       </c>
     </row>
     <row r="100" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10121,7 +10121,7 @@
         <v>54</v>
       </c>
       <c r="H100" s="3">
-        <f>MROUND(G101*1.03, 0.5)</f>
+        <f>MROUND(G100*1.03, 0.5)</f>
       </c>
     </row>
     <row r="101" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10147,7 +10147,7 @@
         <v>169</v>
       </c>
       <c r="H101" s="3">
-        <f>MROUND(G102*1.03, 0.5)</f>
+        <f>MROUND(G101*1.03, 0.5)</f>
       </c>
     </row>
     <row r="102" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10173,7 +10173,7 @@
         <v>269.5</v>
       </c>
       <c r="H102" s="3">
-        <f>MROUND(G103*1.03, 0.5)</f>
+        <f>MROUND(G102*1.03, 0.5)</f>
       </c>
     </row>
     <row r="103" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10199,7 +10199,7 @@
         <v>222</v>
       </c>
       <c r="H103" s="3">
-        <f>MROUND(G104*1.03, 0.5)</f>
+        <f>MROUND(G103*1.03, 0.5)</f>
       </c>
     </row>
     <row r="104" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10225,7 +10225,7 @@
         <v>210</v>
       </c>
       <c r="H104" s="3">
-        <f>MROUND(G105*1.03, 0.5)</f>
+        <f>MROUND(G104*1.03, 0.5)</f>
       </c>
     </row>
     <row r="105" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10251,7 +10251,7 @@
         <v>575</v>
       </c>
       <c r="H105" s="3">
-        <f>MROUND(G106*1.03, 0.5)</f>
+        <f>MROUND(G105*1.03, 0.5)</f>
       </c>
     </row>
     <row r="106" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10277,7 +10277,7 @@
         <v>118.5</v>
       </c>
       <c r="H106" s="3">
-        <f>MROUND(G107*1.03, 0.5)</f>
+        <f>MROUND(G106*1.03, 0.5)</f>
       </c>
     </row>
     <row r="107" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10303,7 +10303,7 @@
         <v>510</v>
       </c>
       <c r="H107" s="3">
-        <f>MROUND(G108*1.03, 0.5)</f>
+        <f>MROUND(G107*1.03, 0.5)</f>
       </c>
     </row>
     <row r="108" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10329,7 +10329,7 @@
         <v>255</v>
       </c>
       <c r="H108" s="3">
-        <f>MROUND(G109*1.03, 0.5)</f>
+        <f>MROUND(G108*1.03, 0.5)</f>
       </c>
     </row>
     <row r="109" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>255</v>
       </c>
       <c r="H109" s="3">
-        <f>MROUND(G110*1.03, 0.5)</f>
+        <f>MROUND(G109*1.03, 0.5)</f>
       </c>
     </row>
     <row r="110" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10381,7 +10381,7 @@
         <v>255</v>
       </c>
       <c r="H110" s="3">
-        <f>MROUND(G111*1.03, 0.5)</f>
+        <f>MROUND(G110*1.03, 0.5)</f>
       </c>
     </row>
     <row r="111" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10407,7 +10407,7 @@
         <v>53</v>
       </c>
       <c r="H111" s="3">
-        <f>MROUND(G112*1.03, 0.5)</f>
+        <f>MROUND(G111*1.03, 0.5)</f>
       </c>
     </row>
     <row r="112" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10433,7 +10433,7 @@
         <v>81.5</v>
       </c>
       <c r="H112" s="3">
-        <f>MROUND(G113*1.03, 0.5)</f>
+        <f>MROUND(G112*1.03, 0.5)</f>
       </c>
     </row>
     <row r="113" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10459,7 +10459,7 @@
         <v>70</v>
       </c>
       <c r="H113" s="3">
-        <f>MROUND(G114*1.03, 0.5)</f>
+        <f>MROUND(G113*1.03, 0.5)</f>
       </c>
     </row>
     <row r="114" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10485,7 +10485,7 @@
         <v>150</v>
       </c>
       <c r="H114" s="3">
-        <f>MROUND(G115*1.03, 0.5)</f>
+        <f>MROUND(G114*1.03, 0.5)</f>
       </c>
     </row>
     <row r="115" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10511,7 +10511,7 @@
         <v>252</v>
       </c>
       <c r="H115" s="3">
-        <f>MROUND(G116*1.03, 0.5)</f>
+        <f>MROUND(G115*1.03, 0.5)</f>
       </c>
     </row>
     <row r="116" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10537,7 +10537,7 @@
         <v>450</v>
       </c>
       <c r="H116" s="3">
-        <f>MROUND(G117*1.03, 0.5)</f>
+        <f>MROUND(G116*1.03, 0.5)</f>
       </c>
     </row>
   </sheetData>
@@ -13705,7 +13705,7 @@
         <v>30</v>
       </c>
       <c r="H66" s="3">
-        <f>MROUND(G65*1.03, 0.5)</f>
+        <f>MROUND(G66*1.03, 0.5)</f>
       </c>
     </row>
     <row r="67" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -13757,7 +13757,7 @@
         <v>64</v>
       </c>
       <c r="H68" s="3">
-        <f>MROUND(G69*1.03, 0.5)</f>
+        <f>MROUND(G68*1.03, 0.5)</f>
       </c>
     </row>
     <row r="69" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -13783,7 +13783,7 @@
         <v>57</v>
       </c>
       <c r="H69" s="3">
-        <f>MROUND(G70*1.03, 0.5)</f>
+        <f>MROUND(G69*1.03, 0.5)</f>
       </c>
     </row>
     <row r="70" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -13809,7 +13809,7 @@
         <v>77</v>
       </c>
       <c r="H70" s="3">
-        <f>MROUND(G71*1.03, 0.5)</f>
+        <f>MROUND(G70*1.03, 0.5)</f>
       </c>
     </row>
     <row r="71" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -13835,7 +13835,7 @@
         <v>77</v>
       </c>
       <c r="H71" s="3">
-        <f>MROUND(G72*1.03, 0.5)</f>
+        <f>MROUND(G71*1.03, 0.5)</f>
       </c>
     </row>
     <row r="72" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -13861,7 +13861,7 @@
         <v>77</v>
       </c>
       <c r="H72" s="3">
-        <f>MROUND(G73*1.03, 0.5)</f>
+        <f>MROUND(G72*1.03, 0.5)</f>
       </c>
     </row>
     <row r="73" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -13887,7 +13887,7 @@
         <v>72</v>
       </c>
       <c r="H73" s="3">
-        <f>MROUND(G74*1.03, 0.5)</f>
+        <f>MROUND(G73*1.03, 0.5)</f>
       </c>
     </row>
     <row r="74" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -13913,7 +13913,7 @@
         <v>144</v>
       </c>
       <c r="H74" s="3">
-        <f>MROUND(G75*1.03, 0.5)</f>
+        <f>MROUND(G74*1.03, 0.5)</f>
       </c>
     </row>
     <row r="75" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -13939,7 +13939,7 @@
         <v>77</v>
       </c>
       <c r="H75" s="3">
-        <f>MROUND(G76*1.03, 0.5)</f>
+        <f>MROUND(G75*1.03, 0.5)</f>
       </c>
     </row>
     <row r="76" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -13965,7 +13965,7 @@
         <v>123.5</v>
       </c>
       <c r="H76" s="3">
-        <f>MROUND(G77*1.03, 0.5)</f>
+        <f>MROUND(G76*1.03, 0.5)</f>
       </c>
     </row>
     <row r="77" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -13991,7 +13991,7 @@
         <v>77</v>
       </c>
       <c r="H77" s="3">
-        <f>MROUND(G78*1.03, 0.5)</f>
+        <f>MROUND(G77*1.03, 0.5)</f>
       </c>
     </row>
     <row r="78" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14017,7 +14017,7 @@
         <v>68.5</v>
       </c>
       <c r="H78" s="3">
-        <f>MROUND(G79*1.03, 0.5)</f>
+        <f>MROUND(G78*1.03, 0.5)</f>
       </c>
     </row>
     <row r="79" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14043,7 +14043,7 @@
         <v>68.5</v>
       </c>
       <c r="H79" s="3">
-        <f>MROUND(G80*1.03, 0.5)</f>
+        <f>MROUND(G79*1.03, 0.5)</f>
       </c>
     </row>
     <row r="80" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14069,7 +14069,7 @@
         <v>177</v>
       </c>
       <c r="H80" s="3">
-        <f>MROUND(G81*1.03, 0.5)</f>
+        <f>MROUND(G80*1.03, 0.5)</f>
       </c>
     </row>
     <row r="81" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14095,7 +14095,7 @@
         <v>75.5</v>
       </c>
       <c r="H81" s="3">
-        <f>MROUND(G82*1.03, 0.5)</f>
+        <f>MROUND(G81*1.03, 0.5)</f>
       </c>
     </row>
     <row r="82" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14121,7 +14121,7 @@
         <v>496</v>
       </c>
       <c r="H82" s="3">
-        <f>MROUND(G83*1.03, 0.5)</f>
+        <f>MROUND(G82*1.03, 0.5)</f>
       </c>
     </row>
     <row r="83" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14147,7 +14147,7 @@
         <v>101</v>
       </c>
       <c r="H83" s="3">
-        <f>MROUND(G84*1.03, 0.5)</f>
+        <f>MROUND(G83*1.03, 0.5)</f>
       </c>
     </row>
     <row r="84" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14173,7 +14173,7 @@
         <v>424</v>
       </c>
       <c r="H84" s="3">
-        <f>MROUND(G85*1.03, 0.5)</f>
+        <f>MROUND(G84*1.03, 0.5)</f>
       </c>
     </row>
     <row r="85" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14199,7 +14199,7 @@
         <v>88</v>
       </c>
       <c r="H85" s="3">
-        <f>MROUND(G86*1.03, 0.5)</f>
+        <f>MROUND(G85*1.03, 0.5)</f>
       </c>
     </row>
     <row r="86" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14225,7 +14225,7 @@
         <v>9</v>
       </c>
       <c r="H86" s="3">
-        <f>MROUND(G87*1.03, 0.5)</f>
+        <f>MROUND(G86*1.03, 0.5)</f>
       </c>
     </row>
     <row r="87" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14251,7 +14251,7 @@
         <v>79.5</v>
       </c>
       <c r="H87" s="3">
-        <f>MROUND(G88*1.03, 0.5)</f>
+        <f>MROUND(G87*1.03, 0.5)</f>
       </c>
     </row>
     <row r="88" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14277,7 +14277,7 @@
         <v>79.5</v>
       </c>
       <c r="H88" s="3">
-        <f>MROUND(G89*1.03, 0.5)</f>
+        <f>MROUND(G88*1.03, 0.5)</f>
       </c>
     </row>
     <row r="89" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14303,7 +14303,7 @@
         <v>79.5</v>
       </c>
       <c r="H89" s="3">
-        <f>MROUND(G90*1.03, 0.5)</f>
+        <f>MROUND(G89*1.03, 0.5)</f>
       </c>
     </row>
     <row r="90" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14329,7 +14329,7 @@
         <v>79.5</v>
       </c>
       <c r="H90" s="3">
-        <f>MROUND(G91*1.03, 0.5)</f>
+        <f>MROUND(G90*1.03, 0.5)</f>
       </c>
     </row>
     <row r="91" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14355,7 +14355,7 @@
         <v>79.5</v>
       </c>
       <c r="H91" s="3">
-        <f>MROUND(G92*1.03, 0.5)</f>
+        <f>MROUND(G91*1.03, 0.5)</f>
       </c>
     </row>
     <row r="92" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14381,7 +14381,7 @@
         <v>79.5</v>
       </c>
       <c r="H92" s="3">
-        <f>MROUND(G93*1.03, 0.5)</f>
+        <f>MROUND(G92*1.03, 0.5)</f>
       </c>
     </row>
     <row r="93" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14407,7 +14407,7 @@
         <v>79.5</v>
       </c>
       <c r="H93" s="3">
-        <f>MROUND(G94*1.03, 0.5)</f>
+        <f>MROUND(G93*1.03, 0.5)</f>
       </c>
     </row>
     <row r="94" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14433,7 +14433,7 @@
         <v>79.5</v>
       </c>
       <c r="H94" s="3">
-        <f>MROUND(G95*1.03, 0.5)</f>
+        <f>MROUND(G94*1.03, 0.5)</f>
       </c>
     </row>
     <row r="95" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14459,7 +14459,7 @@
         <v>79</v>
       </c>
       <c r="H95" s="3">
-        <f>MROUND(G96*1.03, 0.5)</f>
+        <f>MROUND(G95*1.03, 0.5)</f>
       </c>
     </row>
     <row r="96" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14485,7 +14485,7 @@
         <v>45</v>
       </c>
       <c r="H96" s="3">
-        <f>MROUND(G97*1.03, 0.5)</f>
+        <f>MROUND(G96*1.03, 0.5)</f>
       </c>
     </row>
     <row r="97" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14511,7 +14511,7 @@
         <v>60</v>
       </c>
       <c r="H97" s="3">
-        <f>MROUND(G98*1.03, 0.5)</f>
+        <f>MROUND(G97*1.03, 0.5)</f>
       </c>
     </row>
     <row r="98" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14537,7 +14537,7 @@
         <v>81</v>
       </c>
       <c r="H98" s="3">
-        <f>MROUND(G99*1.03, 0.5)</f>
+        <f>MROUND(G98*1.03, 0.5)</f>
       </c>
     </row>
     <row r="99" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14563,7 +14563,7 @@
         <v>81</v>
       </c>
       <c r="H99" s="3">
-        <f>MROUND(G100*1.03, 0.5)</f>
+        <f>MROUND(G99*1.03, 0.5)</f>
       </c>
     </row>
     <row r="100" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14589,7 +14589,7 @@
         <v>30</v>
       </c>
       <c r="H100" s="3">
-        <f>MROUND(G101*1.03, 0.5)</f>
+        <f>MROUND(G100*1.03, 0.5)</f>
       </c>
     </row>
     <row r="101" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14615,7 +14615,7 @@
         <v>25.5</v>
       </c>
       <c r="H101" s="3">
-        <f>MROUND(G102*1.03, 0.5)</f>
+        <f>MROUND(G101*1.03, 0.5)</f>
       </c>
     </row>
     <row r="102" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -14641,7 +14641,7 @@
         <v>27</v>
       </c>
       <c r="H102" s="3">
-        <f>MROUND(G103*1.03, 0.5)</f>
+        <f>MROUND(G102*1.03, 0.5)</f>
       </c>
     </row>
   </sheetData>
@@ -15643,7 +15643,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H92"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -16900,7 +16900,7 @@
         <v>476</v>
       </c>
       <c r="H48" s="3">
-        <f>MROUND(G47*1.03, 0.5)</f>
+        <f>MROUND(G48*1.03, 0.5)</f>
       </c>
     </row>
     <row r="49" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -16926,7 +16926,7 @@
         <v>213.5</v>
       </c>
       <c r="H49" s="3">
-        <f>MROUND(G47*1.03, 0.5)</f>
+        <f>MROUND(G49*1.03, 0.5)</f>
       </c>
     </row>
     <row r="50" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -16952,7 +16952,7 @@
         <v>850.5</v>
       </c>
       <c r="H50" s="3">
-        <f>MROUND(G48*1.03, 0.5)</f>
+        <f>MROUND(G50*1.03, 0.5)</f>
       </c>
     </row>
     <row r="51" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -16978,7 +16978,7 @@
         <v>378.5</v>
       </c>
       <c r="H51" s="3">
-        <f>MROUND(G49*1.03, 0.5)</f>
+        <f>MROUND(G51*1.03, 0.5)</f>
       </c>
     </row>
     <row r="52" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17004,7 +17004,7 @@
         <v>850.5</v>
       </c>
       <c r="H52" s="3">
-        <f>MROUND(G50*1.03, 0.5)</f>
+        <f>MROUND(G52*1.03, 0.5)</f>
       </c>
     </row>
     <row r="53" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17030,7 +17030,7 @@
         <v>378.5</v>
       </c>
       <c r="H53" s="3">
-        <f>MROUND(G51*1.03, 0.5)</f>
+        <f>MROUND(G53*1.03, 0.5)</f>
       </c>
     </row>
     <row r="54" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17056,7 +17056,7 @@
         <v>833.5</v>
       </c>
       <c r="H54" s="3">
-        <f>MROUND(G52*1.03, 0.5)</f>
+        <f>MROUND(G54*1.03, 0.5)</f>
       </c>
     </row>
     <row r="55" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17082,7 +17082,7 @@
         <v>1667</v>
       </c>
       <c r="H55" s="3">
-        <f>MROUND(G53*1.03, 0.5)</f>
+        <f>MROUND(G55*1.03, 0.5)</f>
       </c>
     </row>
     <row r="56" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17108,7 +17108,7 @@
         <v>371</v>
       </c>
       <c r="H56" s="3">
-        <f>MROUND(G54*1.03, 0.5)</f>
+        <f>MROUND(G56*1.03, 0.5)</f>
       </c>
     </row>
     <row r="57" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17134,7 +17134,7 @@
         <v>833.5</v>
       </c>
       <c r="H57" s="3">
-        <f>MROUND(G55*1.03, 0.5)</f>
+        <f>MROUND(G57*1.03, 0.5)</f>
       </c>
     </row>
     <row r="58" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17160,7 +17160,7 @@
         <v>1667</v>
       </c>
       <c r="H58" s="3">
-        <f>MROUND(G56*1.03, 0.5)</f>
+        <f>MROUND(G58*1.03, 0.5)</f>
       </c>
     </row>
     <row r="59" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17186,7 +17186,7 @@
         <v>371</v>
       </c>
       <c r="H59" s="3">
-        <f>MROUND(G57*1.03, 0.5)</f>
+        <f>MROUND(G59*1.03, 0.5)</f>
       </c>
     </row>
     <row r="60" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17212,7 +17212,7 @@
         <v>1950</v>
       </c>
       <c r="H60" s="3">
-        <f>MROUND(G58*1.03, 0.5)</f>
+        <f>MROUND(G60*1.03, 0.5)</f>
       </c>
     </row>
     <row r="61" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17238,7 +17238,7 @@
         <v>458</v>
       </c>
       <c r="H61" s="3">
-        <f>MROUND(G59*1.03, 0.5)</f>
+        <f>MROUND(G61*1.03, 0.5)</f>
       </c>
     </row>
     <row r="62" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17264,7 +17264,7 @@
         <v>1780</v>
       </c>
       <c r="H62" s="3">
-        <f>MROUND(G60*1.03, 0.5)</f>
+        <f>MROUND(G62*1.03, 0.5)</f>
       </c>
     </row>
     <row r="63" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17290,7 +17290,7 @@
         <v>448.5</v>
       </c>
       <c r="H63" s="3">
-        <f>MROUND(G61*1.03, 0.5)</f>
+        <f>MROUND(G63*1.03, 0.5)</f>
       </c>
     </row>
     <row r="64" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17316,7 +17316,7 @@
         <v>433.5</v>
       </c>
       <c r="H64" s="3">
-        <f>MROUND(G62*1.03, 0.5)</f>
+        <f>MROUND(G64*1.03, 0.5)</f>
       </c>
     </row>
     <row r="65" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17342,7 +17342,7 @@
         <v>1720</v>
       </c>
       <c r="H65" s="3">
-        <f>MROUND(G63*1.03, 0.5)</f>
+        <f>MROUND(G65*1.03, 0.5)</f>
       </c>
     </row>
     <row r="66" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17368,7 +17368,7 @@
         <v>1460</v>
       </c>
       <c r="H66" s="3">
-        <f>MROUND(G64*1.03, 0.5)</f>
+        <f>MROUND(G66*1.03, 0.5)</f>
       </c>
     </row>
     <row r="67" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17394,7 +17394,7 @@
         <v>368.5</v>
       </c>
       <c r="H67" s="3">
-        <f>MROUND(G65*1.03, 0.5)</f>
+        <f>MROUND(G67*1.03, 0.5)</f>
       </c>
     </row>
     <row r="68" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17420,7 +17420,7 @@
         <v>145</v>
       </c>
       <c r="H68" s="3">
-        <f>MROUND(G66*1.03, 0.5)</f>
+        <f>MROUND(G68*1.03, 0.5)</f>
       </c>
     </row>
     <row r="69" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17446,7 +17446,7 @@
         <v>75.5</v>
       </c>
       <c r="H69" s="3">
-        <f>MROUND(G67*1.03, 0.5)</f>
+        <f>MROUND(G69*1.03, 0.5)</f>
       </c>
     </row>
     <row r="70" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17472,7 +17472,7 @@
         <v>75.5</v>
       </c>
       <c r="H70" s="3">
-        <f>MROUND(G68*1.03, 0.5)</f>
+        <f>MROUND(G70*1.03, 0.5)</f>
       </c>
     </row>
     <row r="71" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17498,7 +17498,7 @@
         <v>145</v>
       </c>
       <c r="H71" s="3">
-        <f>MROUND(G69*1.03, 0.5)</f>
+        <f>MROUND(G71*1.03, 0.5)</f>
       </c>
     </row>
     <row r="72" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17524,7 +17524,7 @@
         <v>145</v>
       </c>
       <c r="H72" s="3">
-        <f>MROUND(G70*1.03, 0.5)</f>
+        <f>MROUND(G72*1.03, 0.5)</f>
       </c>
     </row>
     <row r="73" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17550,7 +17550,7 @@
         <v>75.5</v>
       </c>
       <c r="H73" s="3">
-        <f>MROUND(G71*1.03, 0.5)</f>
+        <f>MROUND(G73*1.03, 0.5)</f>
       </c>
     </row>
     <row r="74" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17576,7 +17576,7 @@
         <v>166</v>
       </c>
       <c r="H74" s="3">
-        <f>MROUND(G72*1.03, 0.5)</f>
+        <f>MROUND(G74*1.03, 0.5)</f>
       </c>
     </row>
     <row r="75" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17602,7 +17602,7 @@
         <v>83</v>
       </c>
       <c r="H75" s="3">
-        <f>MROUND(G73*1.03, 0.5)</f>
+        <f>MROUND(G75*1.03, 0.5)</f>
       </c>
     </row>
     <row r="76" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17628,7 +17628,7 @@
         <v>145</v>
       </c>
       <c r="H76" s="3">
-        <f>MROUND(G74*1.03, 0.5)</f>
+        <f>MROUND(G76*1.03, 0.5)</f>
       </c>
     </row>
     <row r="77" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17654,7 +17654,7 @@
         <v>75.5</v>
       </c>
       <c r="H77" s="3">
-        <f>MROUND(G75*1.03, 0.5)</f>
+        <f>MROUND(G77*1.03, 0.5)</f>
       </c>
     </row>
     <row r="78" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17680,7 +17680,7 @@
         <v>145</v>
       </c>
       <c r="H78" s="3">
-        <f>MROUND(G76*1.03, 0.5)</f>
+        <f>MROUND(G78*1.03, 0.5)</f>
       </c>
     </row>
     <row r="79" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17706,7 +17706,7 @@
         <v>75.5</v>
       </c>
       <c r="H79" s="3">
-        <f>MROUND(G77*1.03, 0.5)</f>
+        <f>MROUND(G79*1.03, 0.5)</f>
       </c>
     </row>
     <row r="80" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17732,7 +17732,7 @@
         <v>116.5</v>
       </c>
       <c r="H80" s="3">
-        <f>MROUND(G78*1.03, 0.5)</f>
+        <f>MROUND(G80*1.03, 0.5)</f>
       </c>
     </row>
     <row r="81" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17758,7 +17758,7 @@
         <v>1398</v>
       </c>
       <c r="H81" s="3">
-        <f>MROUND(G79*1.03, 0.5)</f>
+        <f>MROUND(G81*1.03, 0.5)</f>
       </c>
     </row>
     <row r="82" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17784,7 +17784,7 @@
         <v>325</v>
       </c>
       <c r="H82" s="3">
-        <f>MROUND(G80*1.03, 0.5)</f>
+        <f>MROUND(G82*1.03, 0.5)</f>
       </c>
     </row>
     <row r="83" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17810,7 +17810,7 @@
         <v>650</v>
       </c>
       <c r="H83" s="3">
-        <f>MROUND(G81*1.03, 0.5)</f>
+        <f>MROUND(G83*1.03, 0.5)</f>
       </c>
     </row>
     <row r="84" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17836,10 +17836,10 @@
         <v>580</v>
       </c>
       <c r="H84" s="3">
-        <f>MROUND(G83*1.03, 0.5)</f>
-      </c>
-    </row>
-    <row r="85" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+        <f>MROUND(G84*1.03, 0.5)</f>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>134</v>
       </c>
@@ -17862,10 +17862,10 @@
         <v>293.5</v>
       </c>
       <c r="H85" s="3">
-        <f>MROUND(G84*1.03, 0.5)</f>
-      </c>
-    </row>
-    <row r="86" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+        <f>MROUND(G85*1.03, 0.5)</f>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
         <v>136</v>
       </c>
@@ -17873,10 +17873,10 @@
         <v>137</v>
       </c>
       <c r="C86" s="3">
-        <v>2330</v>
+        <v>4291</v>
       </c>
       <c r="D86" s="3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E86" s="4" t="s">
         <v>10</v>
@@ -17885,10 +17885,10 @@
         <v>29</v>
       </c>
       <c r="G86" s="3">
-        <v>480</v>
+        <v>528</v>
       </c>
       <c r="H86" s="3">
-        <f>MROUND(G85*1.03, 0.5)</f>
+        <f>MROUND(G86*1.03, 0.5)</f>
       </c>
     </row>
     <row r="87" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17899,74 +17899,74 @@
         <v>137</v>
       </c>
       <c r="C87" s="3">
+        <v>2330</v>
+      </c>
+      <c r="D87" s="3">
+        <v>10</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F87" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G87" s="3">
+        <v>480</v>
+      </c>
+      <c r="H87" s="3">
+        <f>MROUND(G87*1.03, 0.5)</f>
+      </c>
+    </row>
+    <row r="88" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="C88" s="3">
         <v>2385</v>
       </c>
-      <c r="D87" s="3">
-        <v>5</v>
-      </c>
-      <c r="E87" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F87" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G87" s="3">
+      <c r="D88" s="3">
+        <v>5</v>
+      </c>
+      <c r="E88" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F88" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G88" s="3">
         <v>242</v>
       </c>
-      <c r="H87" s="3">
-        <f>MROUND(G86*1.03, 0.5)</f>
-      </c>
-    </row>
-    <row r="88" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A88" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="B88" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="C88" s="3">
-        <v>4540</v>
-      </c>
-      <c r="D88" s="3">
-        <v>10</v>
-      </c>
-      <c r="E88" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F88" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G88" s="3">
-        <v>650</v>
-      </c>
       <c r="H88" s="3">
-        <f>MROUND(G86*1.03, 0.5)</f>
+        <f>MROUND(G88*1.03, 0.5)</f>
       </c>
     </row>
     <row r="89" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" s="4" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C89" s="3">
-        <v>2384</v>
+        <v>4540</v>
       </c>
       <c r="D89" s="3">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E89" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="G89" s="3">
-        <v>187.5</v>
+        <v>650</v>
       </c>
       <c r="H89" s="3">
-        <f>MROUND(G87*1.03, 0.5)</f>
+        <f>MROUND(G89*1.03, 0.5)</f>
       </c>
     </row>
     <row r="90" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -17977,22 +17977,22 @@
         <v>141</v>
       </c>
       <c r="C90" s="3">
-        <v>3851</v>
+        <v>2384</v>
       </c>
       <c r="D90" s="3">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E90" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="G90" s="3">
-        <v>75</v>
+        <v>187.5</v>
       </c>
       <c r="H90" s="3">
-        <f>MROUND(G88*1.03, 0.5)</f>
+        <f>MROUND(G90*1.03, 0.5)</f>
       </c>
     </row>
     <row r="91" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -18003,22 +18003,48 @@
         <v>141</v>
       </c>
       <c r="C91" s="3">
+        <v>3851</v>
+      </c>
+      <c r="D91" s="3">
+        <v>10</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G91" s="3">
+        <v>75</v>
+      </c>
+      <c r="H91" s="3">
+        <f>MROUND(G91*1.03, 0.5)</f>
+      </c>
+    </row>
+    <row r="92" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="C92" s="3">
         <v>2424</v>
       </c>
-      <c r="D91" s="3">
-        <v>5</v>
-      </c>
-      <c r="E91" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F91" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G91" s="3">
+      <c r="D92" s="3">
+        <v>5</v>
+      </c>
+      <c r="E92" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F92" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G92" s="3">
         <v>39.5</v>
       </c>
-      <c r="H91" s="3">
-        <f>MROUND(G89*1.03, 0.5)</f>
+      <c r="H92" s="3">
+        <f>MROUND(G92*1.03, 0.5)</f>
       </c>
     </row>
   </sheetData>
@@ -20002,7 +20028,7 @@
         <v>480</v>
       </c>
       <c r="H48" s="3">
-        <f>MROUND(G47*1.03, 0.5)</f>
+        <f>MROUND(G48*1.03, 0.5)</f>
       </c>
     </row>
     <row r="49" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20028,7 +20054,7 @@
         <v>24</v>
       </c>
       <c r="H49" s="3">
-        <f>MROUND(G48*1.03, 0.5)</f>
+        <f>MROUND(G49*1.03, 0.5)</f>
       </c>
     </row>
     <row r="50" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20054,7 +20080,7 @@
         <v>775</v>
       </c>
       <c r="H50" s="3">
-        <f>MROUND(G49*1.03, 0.5)</f>
+        <f>MROUND(G50*1.03, 0.5)</f>
       </c>
     </row>
     <row r="51" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20080,7 +20106,7 @@
         <v>62</v>
       </c>
       <c r="H51" s="3">
-        <f>MROUND(G50*1.03, 0.5)</f>
+        <f>MROUND(G51*1.03, 0.5)</f>
       </c>
     </row>
     <row r="52" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20106,7 +20132,7 @@
         <v>250</v>
       </c>
       <c r="H52" s="3">
-        <f>MROUND(G51*1.03, 0.5)</f>
+        <f>MROUND(G52*1.03, 0.5)</f>
       </c>
     </row>
     <row r="53" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20132,7 +20158,7 @@
         <v>127</v>
       </c>
       <c r="H53" s="3">
-        <f>MROUND(G52*1.03, 0.5)</f>
+        <f>MROUND(G53*1.03, 0.5)</f>
       </c>
     </row>
     <row r="54" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20158,7 +20184,7 @@
         <v>150</v>
       </c>
       <c r="H54" s="3">
-        <f>MROUND(G53*1.03, 0.5)</f>
+        <f>MROUND(G54*1.03, 0.5)</f>
       </c>
     </row>
     <row r="55" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20184,7 +20210,7 @@
         <v>15</v>
       </c>
       <c r="H55" s="3">
-        <f>MROUND(G54*1.03, 0.5)</f>
+        <f>MROUND(G55*1.03, 0.5)</f>
       </c>
     </row>
     <row r="56" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20210,7 +20236,7 @@
         <v>33</v>
       </c>
       <c r="H56" s="3">
-        <f>MROUND(G55*1.03, 0.5)</f>
+        <f>MROUND(G56*1.03, 0.5)</f>
       </c>
     </row>
     <row r="57" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20236,7 +20262,7 @@
         <v>550</v>
       </c>
       <c r="H57" s="3">
-        <f>MROUND(G56*1.03, 0.5)</f>
+        <f>MROUND(G57*1.03, 0.5)</f>
       </c>
     </row>
     <row r="58" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20262,7 +20288,7 @@
         <v>55</v>
       </c>
       <c r="H58" s="3">
-        <f>MROUND(G57*1.03, 0.5)</f>
+        <f>MROUND(G58*1.03, 0.5)</f>
       </c>
     </row>
     <row r="59" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20288,7 +20314,7 @@
         <v>380</v>
       </c>
       <c r="H59" s="3">
-        <f>MROUND(G58*1.03, 0.5)</f>
+        <f>MROUND(G59*1.03, 0.5)</f>
       </c>
     </row>
     <row r="60" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20314,7 +20340,7 @@
         <v>19</v>
       </c>
       <c r="H60" s="3">
-        <f>MROUND(G59*1.03, 0.5)</f>
+        <f>MROUND(G60*1.03, 0.5)</f>
       </c>
     </row>
     <row r="61" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20340,7 +20366,7 @@
         <v>380</v>
       </c>
       <c r="H61" s="3">
-        <f>MROUND(G60*1.03, 0.5)</f>
+        <f>MROUND(G61*1.03, 0.5)</f>
       </c>
     </row>
     <row r="62" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20366,7 +20392,7 @@
         <v>190</v>
       </c>
       <c r="H62" s="3">
-        <f>MROUND(G61*1.03, 0.5)</f>
+        <f>MROUND(G62*1.03, 0.5)</f>
       </c>
     </row>
     <row r="63" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20392,7 +20418,7 @@
         <v>30</v>
       </c>
       <c r="H63" s="3">
-        <f>MROUND(G62*1.03, 0.5)</f>
+        <f>MROUND(G63*1.03, 0.5)</f>
       </c>
     </row>
     <row r="64" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20418,7 +20444,7 @@
         <v>750</v>
       </c>
       <c r="H64" s="3">
-        <f>MROUND(G63*1.03, 0.5)</f>
+        <f>MROUND(G64*1.03, 0.5)</f>
       </c>
     </row>
     <row r="65" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20444,7 +20470,7 @@
         <v>420</v>
       </c>
       <c r="H65" s="3">
-        <f>MROUND(G64*1.03, 0.5)</f>
+        <f>MROUND(G65*1.03, 0.5)</f>
       </c>
     </row>
     <row r="66" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20470,7 +20496,7 @@
         <v>210</v>
       </c>
       <c r="H66" s="3">
-        <f>MROUND(G65*1.03, 0.5)</f>
+        <f>MROUND(G66*1.03, 0.5)</f>
       </c>
     </row>
     <row r="67" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20496,7 +20522,7 @@
         <v>21</v>
       </c>
       <c r="H67" s="3">
-        <f>MROUND(G66*1.03, 0.5)</f>
+        <f>MROUND(G67*1.03, 0.5)</f>
       </c>
     </row>
     <row r="68" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20522,7 +20548,7 @@
         <v>19</v>
       </c>
       <c r="H68" s="3">
-        <f>MROUND(G67*1.03, 0.5)</f>
+        <f>MROUND(G68*1.03, 0.5)</f>
       </c>
     </row>
     <row r="69" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20548,7 +20574,7 @@
         <v>780</v>
       </c>
       <c r="H69" s="3">
-        <f>MROUND(G68*1.03, 0.5)</f>
+        <f>MROUND(G69*1.03, 0.5)</f>
       </c>
     </row>
     <row r="70" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20574,7 +20600,7 @@
         <v>390</v>
       </c>
       <c r="H70" s="3">
-        <f>MROUND(G69*1.03, 0.5)</f>
+        <f>MROUND(G70*1.03, 0.5)</f>
       </c>
     </row>
     <row r="71" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20600,7 +20626,7 @@
         <v>39</v>
       </c>
       <c r="H71" s="3">
-        <f>MROUND(G70*1.03, 0.5)</f>
+        <f>MROUND(G71*1.03, 0.5)</f>
       </c>
     </row>
     <row r="72" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20626,7 +20652,7 @@
         <v>300</v>
       </c>
       <c r="H72" s="3">
-        <f>MROUND(G71*1.03, 0.5)</f>
+        <f>MROUND(G72*1.03, 0.5)</f>
       </c>
     </row>
     <row r="73" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20652,7 +20678,7 @@
         <v>600</v>
       </c>
       <c r="H73" s="3">
-        <f>MROUND(G72*1.03, 0.5)</f>
+        <f>MROUND(G73*1.03, 0.5)</f>
       </c>
     </row>
     <row r="74" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20678,7 +20704,7 @@
         <v>24</v>
       </c>
       <c r="H74" s="3">
-        <f>MROUND(G73*1.03, 0.5)</f>
+        <f>MROUND(G74*1.03, 0.5)</f>
       </c>
     </row>
     <row r="75" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20704,7 +20730,7 @@
         <v>400</v>
       </c>
       <c r="H75" s="3">
-        <f>MROUND(G74*1.03, 0.5)</f>
+        <f>MROUND(G75*1.03, 0.5)</f>
       </c>
     </row>
     <row r="76" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20730,7 +20756,7 @@
         <v>20</v>
       </c>
       <c r="H76" s="3">
-        <f>MROUND(G75*1.03, 0.5)</f>
+        <f>MROUND(G76*1.03, 0.5)</f>
       </c>
     </row>
     <row r="77" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20756,7 +20782,7 @@
         <v>35</v>
       </c>
       <c r="H77" s="3">
-        <f>MROUND(G76*1.03, 0.5)</f>
+        <f>MROUND(G77*1.03, 0.5)</f>
       </c>
     </row>
     <row r="78" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -20782,7 +20808,7 @@
         <v>350</v>
       </c>
       <c r="H78" s="3">
-        <f>MROUND(G77*1.03, 0.5)</f>
+        <f>MROUND(G78*1.03, 0.5)</f>
       </c>
     </row>
   </sheetData>
@@ -21608,7 +21634,7 @@
         <v>270</v>
       </c>
       <c r="H31" s="3">
-        <f>MROUND(G30*1.03, 0.5)</f>
+        <f>MROUND(G31*1.03, 0.5)</f>
       </c>
     </row>
     <row r="32" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -21634,7 +21660,7 @@
         <v>138.5</v>
       </c>
       <c r="H32" s="3">
-        <f>MROUND(G31*1.03, 0.5)</f>
+        <f>MROUND(G32*1.03, 0.5)</f>
       </c>
     </row>
     <row r="33" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -21660,7 +21686,7 @@
         <v>100</v>
       </c>
       <c r="H33" s="3">
-        <f>MROUND(G32*1.03, 0.5)</f>
+        <f>MROUND(G33*1.03, 0.5)</f>
       </c>
     </row>
     <row r="34" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -21686,7 +21712,7 @@
         <v>52</v>
       </c>
       <c r="H34" s="3">
-        <f>MROUND(G33*1.03, 0.5)</f>
+        <f>MROUND(G34*1.03, 0.5)</f>
       </c>
     </row>
     <row r="35" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -21712,7 +21738,7 @@
         <v>168</v>
       </c>
       <c r="H35" s="3">
-        <f>MROUND(G34*1.03, 0.5)</f>
+        <f>MROUND(G35*1.03, 0.5)</f>
       </c>
     </row>
     <row r="36" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -21738,7 +21764,7 @@
         <v>86</v>
       </c>
       <c r="H36" s="3">
-        <f>MROUND(G35*1.03, 0.5)</f>
+        <f>MROUND(G36*1.03, 0.5)</f>
       </c>
     </row>
     <row r="37" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -21764,7 +21790,7 @@
         <v>160</v>
       </c>
       <c r="H37" s="3">
-        <f>MROUND(G36*1.03, 0.5)</f>
+        <f>MROUND(G37*1.03, 0.5)</f>
       </c>
     </row>
     <row r="38" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -21790,7 +21816,7 @@
         <v>35</v>
       </c>
       <c r="H38" s="3">
-        <f>MROUND(G37*1.03, 0.5)</f>
+        <f>MROUND(G38*1.03, 0.5)</f>
       </c>
     </row>
     <row r="39" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -21816,7 +21842,7 @@
         <v>104.5</v>
       </c>
       <c r="H39" s="3">
-        <f>MROUND(G38*1.03, 0.5)</f>
+        <f>MROUND(G39*1.03, 0.5)</f>
       </c>
     </row>
     <row r="40" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -21842,7 +21868,7 @@
         <v>205</v>
       </c>
       <c r="H40" s="3">
-        <f>MROUND(G39*1.03, 0.5)</f>
+        <f>MROUND(G40*1.03, 0.5)</f>
       </c>
     </row>
     <row r="41" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -21868,7 +21894,7 @@
         <v>66</v>
       </c>
       <c r="H41" s="3">
-        <f>MROUND(G40*1.03, 0.5)</f>
+        <f>MROUND(G41*1.03, 0.5)</f>
       </c>
     </row>
     <row r="42" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -21894,7 +21920,7 @@
         <v>128</v>
       </c>
       <c r="H42" s="3">
-        <f>MROUND(G41*1.03, 0.5)</f>
+        <f>MROUND(G42*1.03, 0.5)</f>
       </c>
     </row>
     <row r="43" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -21920,7 +21946,7 @@
         <v>105</v>
       </c>
       <c r="H43" s="3">
-        <f>MROUND(G42*1.03, 0.5)</f>
+        <f>MROUND(G43*1.03, 0.5)</f>
       </c>
     </row>
     <row r="44" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -21946,7 +21972,7 @@
         <v>90</v>
       </c>
       <c r="H44" s="3">
-        <f>MROUND(G43*1.03, 0.5)</f>
+        <f>MROUND(G44*1.03, 0.5)</f>
       </c>
     </row>
     <row r="45" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -21972,7 +21998,7 @@
         <v>83</v>
       </c>
       <c r="H45" s="3">
-        <f>MROUND(G44*1.03, 0.5)</f>
+        <f>MROUND(G45*1.03, 0.5)</f>
       </c>
     </row>
     <row r="46" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -21998,7 +22024,7 @@
         <v>18.5</v>
       </c>
       <c r="H46" s="3">
-        <f>MROUND(G45*1.03, 0.5)</f>
+        <f>MROUND(G46*1.03, 0.5)</f>
       </c>
     </row>
     <row r="47" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22024,7 +22050,7 @@
         <v>67</v>
       </c>
       <c r="H47" s="3">
-        <f>MROUND(G46*1.03, 0.5)</f>
+        <f>MROUND(G47*1.03, 0.5)</f>
       </c>
     </row>
     <row r="48" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22050,7 +22076,7 @@
         <v>11.5</v>
       </c>
       <c r="H48" s="3">
-        <f>MROUND(G47*1.03, 0.5)</f>
+        <f>MROUND(G48*1.03, 0.5)</f>
       </c>
     </row>
     <row r="49" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22076,7 +22102,7 @@
         <v>96</v>
       </c>
       <c r="H49" s="3">
-        <f>MROUND(G48*1.03, 0.5)</f>
+        <f>MROUND(G49*1.03, 0.5)</f>
       </c>
     </row>
     <row r="50" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22102,7 +22128,7 @@
         <v>22.5</v>
       </c>
       <c r="H50" s="3">
-        <f>MROUND(G49*1.03, 0.5)</f>
+        <f>MROUND(G50*1.03, 0.5)</f>
       </c>
     </row>
     <row r="51" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22128,7 +22154,7 @@
         <v>170</v>
       </c>
       <c r="H51" s="3">
-        <f>MROUND(G50*1.03, 0.5)</f>
+        <f>MROUND(G51*1.03, 0.5)</f>
       </c>
     </row>
     <row r="52" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22154,7 +22180,7 @@
         <v>88</v>
       </c>
       <c r="H52" s="3">
-        <f>MROUND(G51*1.03, 0.5)</f>
+        <f>MROUND(G52*1.03, 0.5)</f>
       </c>
     </row>
     <row r="53" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22180,7 +22206,7 @@
         <v>168</v>
       </c>
       <c r="H53" s="3">
-        <f>MROUND(G52*1.03, 0.5)</f>
+        <f>MROUND(G53*1.03, 0.5)</f>
       </c>
     </row>
     <row r="54" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22206,7 +22232,7 @@
         <v>192</v>
       </c>
       <c r="H54" s="3">
-        <f>MROUND(G53*1.03, 0.5)</f>
+        <f>MROUND(G54*1.03, 0.5)</f>
       </c>
     </row>
     <row r="55" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22232,7 +22258,7 @@
         <v>48</v>
       </c>
       <c r="H55" s="3">
-        <f>MROUND(G54*1.03, 0.5)</f>
+        <f>MROUND(G55*1.03, 0.5)</f>
       </c>
     </row>
     <row r="56" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22258,7 +22284,7 @@
         <v>300</v>
       </c>
       <c r="H56" s="3">
-        <f>MROUND(G55*1.03, 0.5)</f>
+        <f>MROUND(G56*1.03, 0.5)</f>
       </c>
     </row>
     <row r="57" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22284,7 +22310,7 @@
         <v>324</v>
       </c>
       <c r="H57" s="3">
-        <f>MROUND(G56*1.03, 0.5)</f>
+        <f>MROUND(G57*1.03, 0.5)</f>
       </c>
     </row>
     <row r="58" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22310,7 +22336,7 @@
         <v>77</v>
       </c>
       <c r="H58" s="3">
-        <f>MROUND(G57*1.03, 0.5)</f>
+        <f>MROUND(G58*1.03, 0.5)</f>
       </c>
     </row>
     <row r="59" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22336,7 +22362,7 @@
         <v>29</v>
       </c>
       <c r="H59" s="3">
-        <f>MROUND(G58*1.03, 0.5)</f>
+        <f>MROUND(G59*1.03, 0.5)</f>
       </c>
     </row>
     <row r="60" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22362,7 +22388,7 @@
         <v>130</v>
       </c>
       <c r="H60" s="3">
-        <f>MROUND(G59*1.03, 0.5)</f>
+        <f>MROUND(G60*1.03, 0.5)</f>
       </c>
     </row>
     <row r="61" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22388,7 +22414,7 @@
         <v>117</v>
       </c>
       <c r="H61" s="3">
-        <f>MROUND(G60*1.03, 0.5)</f>
+        <f>MROUND(G61*1.03, 0.5)</f>
       </c>
     </row>
     <row r="62" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22414,7 +22440,7 @@
         <v>119</v>
       </c>
       <c r="H62" s="3">
-        <f>MROUND(G61*1.03, 0.5)</f>
+        <f>MROUND(G62*1.03, 0.5)</f>
       </c>
     </row>
     <row r="63" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22440,7 +22466,7 @@
         <v>26</v>
       </c>
       <c r="H63" s="3">
-        <f>MROUND(G62*1.03, 0.5)</f>
+        <f>MROUND(G63*1.03, 0.5)</f>
       </c>
     </row>
     <row r="64" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22466,7 +22492,7 @@
         <v>180</v>
       </c>
       <c r="H64" s="3">
-        <f>MROUND(G63*1.03, 0.5)</f>
+        <f>MROUND(G64*1.03, 0.5)</f>
       </c>
     </row>
     <row r="65" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22492,7 +22518,7 @@
         <v>38</v>
       </c>
       <c r="H65" s="3">
-        <f>MROUND(G64*1.03, 0.5)</f>
+        <f>MROUND(G65*1.03, 0.5)</f>
       </c>
     </row>
     <row r="66" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22518,7 +22544,7 @@
         <v>170</v>
       </c>
       <c r="H66" s="3">
-        <f>MROUND(G65*1.03, 0.5)</f>
+        <f>MROUND(G66*1.03, 0.5)</f>
       </c>
     </row>
     <row r="67" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22544,7 +22570,7 @@
         <v>190</v>
       </c>
       <c r="H67" s="3">
-        <f>MROUND(G66*1.03, 0.5)</f>
+        <f>MROUND(G67*1.03, 0.5)</f>
       </c>
     </row>
     <row r="68" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22570,7 +22596,7 @@
         <v>40</v>
       </c>
       <c r="H68" s="3">
-        <f>MROUND(G67*1.03, 0.5)</f>
+        <f>MROUND(G68*1.03, 0.5)</f>
       </c>
     </row>
     <row r="69" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22596,7 +22622,7 @@
         <v>240</v>
       </c>
       <c r="H69" s="3">
-        <f>MROUND(G68*1.03, 0.5)</f>
+        <f>MROUND(G69*1.03, 0.5)</f>
       </c>
     </row>
     <row r="70" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22622,7 +22648,7 @@
         <v>123.5</v>
       </c>
       <c r="H70" s="3">
-        <f>MROUND(G69*1.03, 0.5)</f>
+        <f>MROUND(G70*1.03, 0.5)</f>
       </c>
     </row>
     <row r="71" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22648,7 +22674,7 @@
         <v>360</v>
       </c>
       <c r="H71" s="3">
-        <f>MROUND(G70*1.03, 0.5)</f>
+        <f>MROUND(G71*1.03, 0.5)</f>
       </c>
     </row>
     <row r="72" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -22674,7 +22700,7 @@
         <v>183.5</v>
       </c>
       <c r="H72" s="3">
-        <f>MROUND(G71*1.03, 0.5)</f>
+        <f>MROUND(G72*1.03, 0.5)</f>
       </c>
     </row>
   </sheetData>
@@ -23916,7 +23942,7 @@
         <v>115</v>
       </c>
       <c r="H47" s="3">
-        <f>MROUND(G46*1.03, 0.5)</f>
+        <f>MROUND(G47*1.03, 0.5)</f>
       </c>
     </row>
     <row r="48" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -23942,7 +23968,7 @@
         <v>26</v>
       </c>
       <c r="H48" s="3">
-        <f>MROUND(G47*1.03, 0.5)</f>
+        <f>MROUND(G48*1.03, 0.5)</f>
       </c>
     </row>
     <row r="49" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -23968,7 +23994,7 @@
         <v>170</v>
       </c>
       <c r="H49" s="3">
-        <f>MROUND(G48*1.03, 0.5)</f>
+        <f>MROUND(G49*1.03, 0.5)</f>
       </c>
     </row>
     <row r="50" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -23994,7 +24020,7 @@
         <v>31.5</v>
       </c>
       <c r="H50" s="3">
-        <f>MROUND(G49*1.03, 0.5)</f>
+        <f>MROUND(G50*1.03, 0.5)</f>
       </c>
     </row>
     <row r="51" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24020,7 +24046,7 @@
         <v>320</v>
       </c>
       <c r="H51" s="3">
-        <f>MROUND(G50*1.03, 0.5)</f>
+        <f>MROUND(G51*1.03, 0.5)</f>
       </c>
     </row>
     <row r="52" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24046,7 +24072,7 @@
         <v>55.5</v>
       </c>
       <c r="H52" s="3">
-        <f>MROUND(G51*1.03, 0.5)</f>
+        <f>MROUND(G52*1.03, 0.5)</f>
       </c>
     </row>
     <row r="53" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24072,7 +24098,7 @@
         <v>362.5</v>
       </c>
       <c r="H53" s="3">
-        <f>MROUND(G52*1.03, 0.5)</f>
+        <f>MROUND(G53*1.03, 0.5)</f>
       </c>
     </row>
     <row r="54" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24098,7 +24124,7 @@
         <v>74.5</v>
       </c>
       <c r="H54" s="3">
-        <f>MROUND(G53*1.03, 0.5)</f>
+        <f>MROUND(G54*1.03, 0.5)</f>
       </c>
     </row>
     <row r="55" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24124,7 +24150,7 @@
         <v>255</v>
       </c>
       <c r="H55" s="3">
-        <f>MROUND(G54*1.03, 0.5)</f>
+        <f>MROUND(G55*1.03, 0.5)</f>
       </c>
     </row>
     <row r="56" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24150,7 +24176,7 @@
         <v>212.5</v>
       </c>
       <c r="H56" s="3">
-        <f>MROUND(G55*1.03, 0.5)</f>
+        <f>MROUND(G56*1.03, 0.5)</f>
       </c>
     </row>
     <row r="57" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24176,7 +24202,7 @@
         <v>44.5</v>
       </c>
       <c r="H57" s="3">
-        <f>MROUND(G56*1.03, 0.5)</f>
+        <f>MROUND(G57*1.03, 0.5)</f>
       </c>
     </row>
     <row r="58" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24202,7 +24228,7 @@
         <v>350</v>
       </c>
       <c r="H58" s="3">
-        <f>MROUND(G57*1.03, 0.5)</f>
+        <f>MROUND(G58*1.03, 0.5)</f>
       </c>
     </row>
     <row r="59" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24228,7 +24254,7 @@
         <v>175</v>
       </c>
       <c r="H59" s="3">
-        <f>MROUND(G58*1.03, 0.5)</f>
+        <f>MROUND(G59*1.03, 0.5)</f>
       </c>
     </row>
     <row r="60" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24254,7 +24280,7 @@
         <v>32</v>
       </c>
       <c r="H60" s="3">
-        <f>MROUND(G59*1.03, 0.5)</f>
+        <f>MROUND(G60*1.03, 0.5)</f>
       </c>
     </row>
     <row r="61" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24280,7 +24306,7 @@
         <v>275</v>
       </c>
       <c r="H61" s="3">
-        <f>MROUND(G60*1.03, 0.5)</f>
+        <f>MROUND(G61*1.03, 0.5)</f>
       </c>
     </row>
     <row r="62" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24306,7 +24332,7 @@
         <v>57</v>
       </c>
       <c r="H62" s="3">
-        <f>MROUND(G61*1.03, 0.5)</f>
+        <f>MROUND(G62*1.03, 0.5)</f>
       </c>
     </row>
     <row r="63" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24332,7 +24358,7 @@
         <v>280</v>
       </c>
       <c r="H63" s="3">
-        <f>MROUND(G62*1.03, 0.5)</f>
+        <f>MROUND(G63*1.03, 0.5)</f>
       </c>
     </row>
     <row r="64" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24358,7 +24384,7 @@
         <v>48.5</v>
       </c>
       <c r="H64" s="3">
-        <f>MROUND(G63*1.03, 0.5)</f>
+        <f>MROUND(G64*1.03, 0.5)</f>
       </c>
     </row>
     <row r="65" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24384,7 +24410,7 @@
         <v>375</v>
       </c>
       <c r="H65" s="3">
-        <f>MROUND(G64*1.03, 0.5)</f>
+        <f>MROUND(G65*1.03, 0.5)</f>
       </c>
     </row>
     <row r="66" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24410,7 +24436,7 @@
         <v>64.5</v>
       </c>
       <c r="H66" s="3">
-        <f>MROUND(G65*1.03, 0.5)</f>
+        <f>MROUND(G66*1.03, 0.5)</f>
       </c>
     </row>
     <row r="67" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24436,7 +24462,7 @@
         <v>330</v>
       </c>
       <c r="H67" s="3">
-        <f>MROUND(G66*1.03, 0.5)</f>
+        <f>MROUND(G67*1.03, 0.5)</f>
       </c>
     </row>
     <row r="68" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24462,7 +24488,7 @@
         <v>57</v>
       </c>
       <c r="H68" s="3">
-        <f>MROUND(G67*1.03, 0.5)</f>
+        <f>MROUND(G68*1.03, 0.5)</f>
       </c>
     </row>
     <row r="69" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24488,7 +24514,7 @@
         <v>237.5</v>
       </c>
       <c r="H69" s="3">
-        <f>MROUND(G68*1.03, 0.5)</f>
+        <f>MROUND(G69*1.03, 0.5)</f>
       </c>
     </row>
     <row r="70" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24514,7 +24540,7 @@
         <v>50.5</v>
       </c>
       <c r="H70" s="3">
-        <f>MROUND(G69*1.03, 0.5)</f>
+        <f>MROUND(G70*1.03, 0.5)</f>
       </c>
     </row>
     <row r="71" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24540,7 +24566,7 @@
         <v>312.5</v>
       </c>
       <c r="H71" s="3">
-        <f>MROUND(G70*1.03, 0.5)</f>
+        <f>MROUND(G71*1.03, 0.5)</f>
       </c>
     </row>
     <row r="72" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24566,7 +24592,7 @@
         <v>64.5</v>
       </c>
       <c r="H72" s="3">
-        <f>MROUND(G71*1.03, 0.5)</f>
+        <f>MROUND(G72*1.03, 0.5)</f>
       </c>
     </row>
     <row r="73" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24592,7 +24618,7 @@
         <v>262.5</v>
       </c>
       <c r="H73" s="3">
-        <f>MROUND(G72*1.03, 0.5)</f>
+        <f>MROUND(G73*1.03, 0.5)</f>
       </c>
     </row>
     <row r="74" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24618,7 +24644,7 @@
         <v>55.5</v>
       </c>
       <c r="H74" s="3">
-        <f>MROUND(G73*1.03, 0.5)</f>
+        <f>MROUND(G74*1.03, 0.5)</f>
       </c>
     </row>
     <row r="75" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24644,7 +24670,7 @@
         <v>162.5</v>
       </c>
       <c r="H75" s="3">
-        <f>MROUND(G74*1.03, 0.5)</f>
+        <f>MROUND(G75*1.03, 0.5)</f>
       </c>
     </row>
     <row r="76" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24670,7 +24696,7 @@
         <v>35.5</v>
       </c>
       <c r="H76" s="3">
-        <f>MROUND(G75*1.03, 0.5)</f>
+        <f>MROUND(G76*1.03, 0.5)</f>
       </c>
     </row>
     <row r="77" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24696,7 +24722,7 @@
         <v>179</v>
       </c>
       <c r="H77" s="3">
-        <f>MROUND(G76*1.03, 0.5)</f>
+        <f>MROUND(G77*1.03, 0.5)</f>
       </c>
     </row>
     <row r="78" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24722,7 +24748,7 @@
         <v>358</v>
       </c>
       <c r="H78" s="3">
-        <f>MROUND(G77*1.03, 0.5)</f>
+        <f>MROUND(G78*1.03, 0.5)</f>
       </c>
     </row>
     <row r="79" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24748,7 +24774,7 @@
         <v>42.5</v>
       </c>
       <c r="H79" s="3">
-        <f>MROUND(G78*1.03, 0.5)</f>
+        <f>MROUND(G79*1.03, 0.5)</f>
       </c>
     </row>
     <row r="80" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24774,7 +24800,7 @@
         <v>544</v>
       </c>
       <c r="H80" s="3">
-        <f>MROUND(G79*1.03, 0.5)</f>
+        <f>MROUND(G80*1.03, 0.5)</f>
       </c>
     </row>
     <row r="81" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24800,7 +24826,7 @@
         <v>272</v>
       </c>
       <c r="H81" s="3">
-        <f>MROUND(G80*1.03, 0.5)</f>
+        <f>MROUND(G81*1.03, 0.5)</f>
       </c>
     </row>
     <row r="82" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24826,7 +24852,7 @@
         <v>63</v>
       </c>
       <c r="H82" s="3">
-        <f>MROUND(G81*1.03, 0.5)</f>
+        <f>MROUND(G82*1.03, 0.5)</f>
       </c>
     </row>
     <row r="83" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24852,7 +24878,7 @@
         <v>52</v>
       </c>
       <c r="H83" s="3">
-        <f>MROUND(G82*1.03, 0.5)</f>
+        <f>MROUND(G83*1.03, 0.5)</f>
       </c>
     </row>
     <row r="84" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24878,7 +24904,7 @@
         <v>182</v>
       </c>
       <c r="H84" s="3">
-        <f>MROUND(G83*1.03, 0.5)</f>
+        <f>MROUND(G84*1.03, 0.5)</f>
       </c>
     </row>
     <row r="85" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24904,7 +24930,7 @@
         <v>350</v>
       </c>
       <c r="H85" s="3">
-        <f>MROUND(G84*1.03, 0.5)</f>
+        <f>MROUND(G85*1.03, 0.5)</f>
       </c>
     </row>
     <row r="86" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24930,7 +24956,7 @@
         <v>700</v>
       </c>
       <c r="H86" s="3">
-        <f>MROUND(G85*1.03, 0.5)</f>
+        <f>MROUND(G86*1.03, 0.5)</f>
       </c>
     </row>
     <row r="87" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24956,7 +24982,7 @@
         <v>106</v>
       </c>
       <c r="H87" s="3">
-        <f>MROUND(G86*1.03, 0.5)</f>
+        <f>MROUND(G87*1.03, 0.5)</f>
       </c>
     </row>
     <row r="88" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24982,7 +25008,7 @@
         <v>87</v>
       </c>
       <c r="H88" s="3">
-        <f>MROUND(G87*1.03, 0.5)</f>
+        <f>MROUND(G88*1.03, 0.5)</f>
       </c>
     </row>
     <row r="89" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -25008,7 +25034,7 @@
         <v>85</v>
       </c>
       <c r="H89" s="3">
-        <f>MROUND(G88*1.03, 0.5)</f>
+        <f>MROUND(G89*1.03, 0.5)</f>
       </c>
     </row>
     <row r="90" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -25034,7 +25060,7 @@
         <v>21</v>
       </c>
       <c r="H90" s="3">
-        <f>MROUND(G89*1.03, 0.5)</f>
+        <f>MROUND(G90*1.03, 0.5)</f>
       </c>
     </row>
     <row r="91" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -25060,7 +25086,7 @@
         <v>110</v>
       </c>
       <c r="H91" s="3">
-        <f>MROUND(G90*1.03, 0.5)</f>
+        <f>MROUND(G91*1.03, 0.5)</f>
       </c>
     </row>
     <row r="92" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -25086,7 +25112,7 @@
         <v>25</v>
       </c>
       <c r="H92" s="3">
-        <f>MROUND(G91*1.03, 0.5)</f>
+        <f>MROUND(G92*1.03, 0.5)</f>
       </c>
     </row>
     <row r="93" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -25727,7 +25753,7 @@
         <v>12</v>
       </c>
       <c r="G22" s="3">
-        <v>170</v>
+        <v>140</v>
       </c>
       <c r="H22" s="3">
         <f>MROUND(G22*1.03, 0.5)</f>
@@ -28018,7 +28044,7 @@
         <v>170</v>
       </c>
       <c r="H110" s="3">
-        <f>MROUND(G108*1.03, 0.5)</f>
+        <f>MROUND(G110*1.03, 0.5)</f>
       </c>
     </row>
     <row r="111" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -28044,7 +28070,7 @@
         <v>88</v>
       </c>
       <c r="H111" s="3">
-        <f>MROUND(G108*1.03, 0.5)</f>
+        <f>MROUND(G111*1.03, 0.5)</f>
       </c>
     </row>
     <row r="112" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -28070,7 +28096,7 @@
         <v>1175</v>
       </c>
       <c r="H112" s="3">
-        <f>MROUND(G110*1.03, 0.5)</f>
+        <f>MROUND(G112*1.03, 0.5)</f>
       </c>
     </row>
     <row r="113" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -28096,7 +28122,7 @@
         <v>235</v>
       </c>
       <c r="H113" s="3">
-        <f>MROUND(G111*1.03, 0.5)</f>
+        <f>MROUND(G113*1.03, 0.5)</f>
       </c>
     </row>
     <row r="114" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -28122,7 +28148,7 @@
         <v>73.5</v>
       </c>
       <c r="H114" s="3">
-        <f>MROUND(G112*1.03, 0.5)</f>
+        <f>MROUND(G114*1.03, 0.5)</f>
       </c>
     </row>
     <row r="115" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -28148,7 +28174,7 @@
         <v>200</v>
       </c>
       <c r="H115" s="3">
-        <f>MROUND(G113*1.03, 0.5)</f>
+        <f>MROUND(G115*1.03, 0.5)</f>
       </c>
     </row>
     <row r="116" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -28174,7 +28200,7 @@
         <v>20</v>
       </c>
       <c r="H116" s="3">
-        <f>MROUND(G114*1.03, 0.5)</f>
+        <f>MROUND(G116*1.03, 0.5)</f>
       </c>
     </row>
     <row r="117" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -28200,7 +28226,7 @@
         <v>90</v>
       </c>
       <c r="H117" s="3">
-        <f>MROUND(G115*1.03, 0.5)</f>
+        <f>MROUND(G117*1.03, 0.5)</f>
       </c>
     </row>
     <row r="118" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -28226,7 +28252,7 @@
         <v>84</v>
       </c>
       <c r="H118" s="3">
-        <f>MROUND(G116*1.03, 0.5)</f>
+        <f>MROUND(G118*1.03, 0.5)</f>
       </c>
     </row>
   </sheetData>

</xml_diff>